<commit_message>
Fix range clear method
The clear should set format to the worksheet format, but former code only
changed formatting properties. Things like what is included or cell style
were not changed.

That caused duplicate xf records in styles part (should use default
format, used a new one).
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotCacheWithoutSourceData-output.xlsx
+++ b/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotCacheWithoutSourceData-output.xlsx
@@ -52,186 +52,174 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2 xr">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="2" x14ac:knownFonts="1">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="10">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:bottom>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right/>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:bottom>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="65"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color indexed="65"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFABABAB"/>
-      </x:bottom>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="2">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="11">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="10">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFABABAB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFABABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFABABAB"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFABABAB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
-</x:styleSheet>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>